<commit_message>
feat: convert panel.js to TypeScript, add cell editing, write marketplace README
- Convert media/panel.js → src/webview/panel.ts with full type annotations
- Add tsconfig.webview.json (DOM + ESNext) for webview TypeScript target
- Update esbuild to build both extension host and webview panel as separate contexts
- Add check-types:webview and watch:tsc-webview npm scripts
- Add src/core/fastxlsx/writeCellValue.ts: write cell value to local .xlsx via fastxlsx
- Add editCell webview message: double-click any non-readonly cell to edit inline
  - Enter/Tab commits, Escape cancels; ghost cells and read-only files are blocked
  - Extension writes value and reloads diff view on commit
- Rewrite README.md as marketplace documentation with feature list, usage guide, settings table, and Git difftool setup
</commit_message>
<xml_diff>
--- a/res/item.xlsx
+++ b/res/item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypess/Desktop/Github/vscode-xlsx-diff/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E13251E-55ED-44B9-A65E-8ECF2B42EF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBDBD03B-7144-D143-A19D-D55B6C782748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30780" yWindow="1335" windowWidth="28395" windowHeight="18750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="2" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="125">
   <si>
     <t>id</t>
   </si>
@@ -505,24 +505,27 @@
   <si>
     <t>$.length == arr1.length</t>
     <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>[2,3]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -556,13 +559,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -570,7 +573,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -760,7 +763,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
   <dxfs count="6">
@@ -1090,18 +1093,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="3" max="3" width="24.125" customWidth="1"/>
-    <col min="4" max="4" width="21.125" customWidth="1"/>
-    <col min="5" max="5" width="20.375" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.625" customWidth="1"/>
-    <col min="8" max="8" width="18.375" style="16" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" s="28" t="s">
         <v>110</v>
       </c>
@@ -1113,7 +1116,7 @@
       <c r="G1" s="29"/>
       <c r="H1" s="29"/>
     </row>
-    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="16">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1139,7 +1142,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="16">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -1165,7 +1168,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="16">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1177,7 +1180,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="16">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1203,7 +1206,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="16">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1219,7 +1222,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="16">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -1239,7 +1242,7 @@
       </c>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="16">
       <c r="A8" s="1" t="s">
         <v>65</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="16">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -1287,7 +1290,7 @@
       </c>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="16">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1309,7 +1312,7 @@
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="16">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1331,7 +1334,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="16">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -1357,7 +1360,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="16">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -1381,7 +1384,7 @@
       </c>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="16">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -1405,7 +1408,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="16">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -1427,7 +1430,7 @@
       </c>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="16">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -1449,7 +1452,7 @@
       </c>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="16">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
@@ -1471,7 +1474,7 @@
       </c>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="16">
       <c r="A18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1506,22 +1509,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="6.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="13.125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="90.875" style="10" customWidth="1"/>
-    <col min="10" max="10" width="24.375" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="90.83203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="24.33203125" style="10" customWidth="1"/>
     <col min="11" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1585,7 +1588,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1603,7 +1606,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1635,7 +1638,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="34">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1667,7 +1670,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="4">
         <v>10101</v>
       </c>
@@ -1699,7 +1702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="4">
         <v>10102</v>
       </c>
@@ -1719,7 +1722,7 @@
         <v>71</v>
       </c>
       <c r="G7" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>35</v>
@@ -1731,7 +1734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="4">
         <v>10103</v>
       </c>
@@ -1763,7 +1766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="4">
         <v>10104</v>
       </c>
@@ -1795,7 +1798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="4">
         <v>10105</v>
       </c>
@@ -1827,7 +1830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="4">
         <v>10201</v>
       </c>
@@ -1857,7 +1860,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="4">
         <v>10202</v>
       </c>
@@ -1887,7 +1890,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="4">
         <v>10203</v>
       </c>
@@ -1931,14 +1934,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B4D15F-7CDD-ED40-889B-A4868E886B80}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" style="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1955,7 +1958,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1972,7 +1975,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1981,7 +1984,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1998,7 +2001,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="17">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -2009,7 +2012,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -2026,7 +2029,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -2036,10 +2039,12 @@
       <c r="C7" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="27"/>
+      <c r="D7" s="27" t="s">
+        <v>124</v>
+      </c>
       <c r="E7" s="27"/>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -2052,7 +2057,7 @@
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="4">
         <v>4</v>
       </c>
@@ -2065,7 +2070,7 @@
       <c r="D9" s="27"/>
       <c r="E9" s="27"/>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="4">
         <v>5</v>
       </c>
@@ -2074,7 +2079,7 @@
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
     </row>
-    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="16">
       <c r="A11" s="4">
         <v>6</v>
       </c>
@@ -2087,7 +2092,7 @@
       <c r="D11" s="27"/>
       <c r="E11" s="27"/>
     </row>
-    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="16">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -2100,7 +2105,7 @@
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
     </row>
-    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="16">
       <c r="A13" s="4">
         <v>8</v>
       </c>
@@ -2125,19 +2130,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E27B46D-4699-4B1C-B2B1-8A327D06725E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="25" customFormat="1">
       <c r="A1" s="26" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="7" t="s">
         <v>118</v>
       </c>
@@ -2154,7 +2159,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2171,7 +2176,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2182,7 +2187,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2199,7 +2204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2212,7 +2217,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
@@ -2229,7 +2234,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
@@ -2246,7 +2251,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
@@ -2263,7 +2268,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
@@ -2292,19 +2297,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E541871-473E-3747-A4FF-7005DDAE5E45}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="25" customFormat="1">
       <c r="A1" s="26" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2321,7 +2326,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2338,7 +2343,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2349,7 +2354,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2366,7 +2371,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2379,7 +2384,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
@@ -2396,7 +2401,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
@@ -2413,7 +2418,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
@@ -2430,7 +2435,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
@@ -2459,19 +2464,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D10B9FB-C914-9E4D-9ED5-4AA283A47ADC}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="25" customFormat="1">
       <c r="A1" s="26" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2488,7 +2493,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2505,7 +2510,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2516,7 +2521,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2533,7 +2538,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2546,7 +2551,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
@@ -2563,7 +2568,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
@@ -2580,7 +2585,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
@@ -2597,7 +2602,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
@@ -2626,19 +2631,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA9512F-15D7-C04B-B65B-D43362DB2865}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="25" customFormat="1">
       <c r="A1" s="26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2655,7 +2660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2672,7 +2677,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2683,7 +2688,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2700,7 +2705,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2713,7 +2718,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
@@ -2730,7 +2735,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
@@ -2747,7 +2752,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
@@ -2764,7 +2769,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
@@ -2793,9 +2798,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBB972E-C927-480C-A467-3665FD9F033A}">
   <dimension ref="B2"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2">
       <c r="B2" s="22" t="s">
         <v>98</v>
       </c>

</xml_diff>